<commit_message>
for the Frequency Conversion paper
Create exogenous variables for the projection exercise in the Frequency Conversion Paper based on the Wealth Module's personal pension participation.
</commit_message>
<xml_diff>
--- a/input/DatabaseCountryYear.xlsx
+++ b/input/DatabaseCountryYear.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="9">
   <si>
     <t>Country</t>
   </si>
@@ -30,6 +30,15 @@
   </si>
   <si>
     <t>2011</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>2021</t>
+  </si>
+  <si>
+    <t>2017</t>
   </si>
 </sst>
 </file>
@@ -90,7 +99,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>